<commit_message>
docs(costos): hoja 00 usa la misma tasa COP/USD que el sistema (3.048,12)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Costo360_Costos_Operativos_Mensuales.xlsx
+++ b/docs/Costo360_Costos_Operativos_Mensuales.xlsx
@@ -303,7 +303,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -433,6 +433,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -896,8 +897,15 @@
           <t>Tasa de cambio COP por USD (editable)</t>
         </is>
       </c>
-      <c r="E5" s="46" t="n">
-        <v>4000</v>
+      <c r="E5" s="61" t="n">
+        <v>3048.12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Misma tasa que usa el sistema (backend/services/consumo_service.py TRM_COP_USD). Si cambias una, cambia la otra. Los costos fijos que usa el agente viven en la tabla metricas.costos_fijos de la base de datos.</t>
+        </is>
       </c>
     </row>
     <row r="7">

</xml_diff>